<commit_message>
Medals: Adjust columns for better printing on weird USAW laptop
</commit_message>
<xml_diff>
--- a/local/templates/medals/Medals.xlsx
+++ b/local/templates/medals/Medals.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/Misc/usaw-owlcms/local/templates/medals/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/templates/medals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{364734E5-81ED-924A-BAF3-FC73EAD501B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15BEDB7F-62BB-FE42-A476-258EE67753EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5460" yWindow="5000" windowWidth="31800" windowHeight="19000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -144,16 +144,61 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>jx:each(</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">jx:each(
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+          </rPr>
+          <t xml:space="preserve">  items="group.items"
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+          </rPr>
+          <t xml:space="preserve">  var="lift"
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+          </rPr>
+          <t xml:space="preserve">  groupBy="lift.rankingText"
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+          </rPr>
+          <t xml:space="preserve">  lastCell="D8"
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+          </rPr>
+          <t xml:space="preserve">)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Aptos Narrow"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -163,111 +208,6 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">  items="group.items"</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">  var="lift"</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">  groupBy="lift.rankingText"</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">  lastCell="D8"</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>)</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Aptos Narrow"/>
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">jx:if(
@@ -287,7 +227,6 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Aptos Narrow"/>
-            <scheme val="minor"/>
           </rPr>
           <t>CATEGORY_SCORE</t>
         </r>
@@ -478,13 +417,12 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -519,14 +457,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -868,19 +806,18 @@
   <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="40.6640625" customWidth="1"/>
-    <col min="3" max="3" width="46.6640625" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="37" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
@@ -889,12 +826,12 @@
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="1:4" ht="31" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
@@ -903,12 +840,12 @@
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" ht="24" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="1"/>

</xml_diff>